<commit_message>
implement policy management module with file upload and CRUD support
</commit_message>
<xml_diff>
--- a/src/routes/PolicyManagement/uploadPolicyManagementCsv/policyData-6a3e738df809400f86d417a7 (1).xlsx
+++ b/src/routes/PolicyManagement/uploadPolicyManagementCsv/policyData-6a3e738df809400f86d417a7 (1).xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:CW3"/>
+  <dimension ref="A1:CW8"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -713,7 +713,7 @@
         <v>retail</v>
       </c>
       <c r="C2" t="str">
-        <v>KISHAN</v>
+        <v>GLASS GUARD INDIA PRIVATE LIMITED</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -725,25 +725,25 @@
         <v/>
       </c>
       <c r="G2" t="str">
-        <v>test</v>
+        <v>JP INSURANCE BROKERS PVT LTD</v>
       </c>
       <c r="H2" t="str">
-        <v>jhgfcdxzsxdcf</v>
+        <v>NAGPUR</v>
       </c>
       <c r="I2" t="str">
-        <v>Mr.</v>
+        <v>M/S</v>
       </c>
       <c r="J2" t="str">
-        <v>KISHAN</v>
+        <v>GLASS GUARD INDIA PRIVATE LIMITED</v>
       </c>
       <c r="K2" t="str">
-        <v>8805881253</v>
+        <v>9373120261</v>
       </c>
       <c r="L2" t="str">
         <v/>
       </c>
       <c r="M2" t="str">
-        <v>BAJAJ ALLIANZ GENERAL INSURANCE CO. LTD.</v>
+        <v>GENERALI CENTRAL INSURANCE COMPANY LIMITED</v>
       </c>
       <c r="N2" t="str">
         <v/>
@@ -764,70 +764,70 @@
         <v>MOTOR</v>
       </c>
       <c r="T2" t="str">
-        <v>TWO WHEELER</v>
+        <v>COMMERCIAL VEHICLE (GOODS CARRYING)</v>
       </c>
       <c r="U2" t="str">
         <v/>
       </c>
       <c r="V2" t="str">
-        <v/>
+        <v>GENERALI CENTRAL INSURANCE COMPANY LIMITED</v>
       </c>
       <c r="W2" t="str">
-        <v>test</v>
+        <v>JP INSURANCE BROKER PVT. LTD</v>
       </c>
       <c r="X2" t="str">
-        <v>test</v>
+        <v>NAGPUR</v>
       </c>
       <c r="Y2" t="str">
         <v>YEARLY</v>
       </c>
       <c r="Z2" s="1">
-        <v>45839</v>
+        <v>46216</v>
       </c>
       <c r="AA2" s="1">
-        <v>46203</v>
+        <v>46580</v>
       </c>
       <c r="AB2" t="str">
-        <v>714</v>
+        <v>16099</v>
       </c>
       <c r="AC2">
-        <v>18</v>
+        <v>5</v>
       </c>
       <c r="AD2" t="str">
-        <v>128.51999999999998</v>
+        <v>804.95</v>
       </c>
       <c r="AE2" t="str">
-        <v>714</v>
+        <v>16099</v>
       </c>
       <c r="AF2" t="str">
         <v>YEARLY</v>
       </c>
       <c r="AG2" s="1">
-        <v>45839</v>
+        <v>46216</v>
       </c>
       <c r="AH2" s="1">
-        <v>46203</v>
+        <v>46580</v>
       </c>
       <c r="AI2" t="str">
-        <v>39</v>
+        <v>4591</v>
       </c>
       <c r="AJ2">
         <v>18</v>
       </c>
       <c r="AK2" t="str">
-        <v>7.02</v>
+        <v>826.38</v>
       </c>
       <c r="AL2" t="str">
-        <v>39</v>
+        <v>4591</v>
       </c>
       <c r="AM2" t="str">
-        <v>123456789</v>
+        <v>132/02/17/0727/MTP/1010550083</v>
       </c>
       <c r="AN2" s="1">
-        <v>46203</v>
+        <v>46580</v>
       </c>
       <c r="AO2">
-        <v>50000</v>
+        <v>713336</v>
       </c>
       <c r="AP2" t="str">
         <v>RENEWAL</v>
@@ -842,10 +842,10 @@
         <v/>
       </c>
       <c r="AU2" s="1">
-        <v>46204</v>
+        <v>46216</v>
       </c>
       <c r="AV2" s="1">
-        <v>46568</v>
+        <v>46580</v>
       </c>
       <c r="AW2" t="str">
         <v/>
@@ -854,7 +854,7 @@
         <v/>
       </c>
       <c r="AZ2">
-        <v>753</v>
+        <v>20690</v>
       </c>
       <c r="BA2" t="str">
         <v/>
@@ -872,10 +872,10 @@
         <v/>
       </c>
       <c r="BF2">
-        <v>135.54</v>
+        <v>1631.33</v>
       </c>
       <c r="BG2" t="str">
-        <v>888.54</v>
+        <v>22321.33</v>
       </c>
       <c r="BH2" t="str">
         <v/>
@@ -893,31 +893,31 @@
         <v/>
       </c>
       <c r="BN2" t="str">
-        <v>753</v>
+        <v>20690</v>
       </c>
       <c r="BO2" t="str">
-        <v xml:space="preserve">HONDA </v>
+        <v xml:space="preserve">ASHOK LEYLAND </v>
       </c>
       <c r="BP2" t="str">
-        <v xml:space="preserve">ACTIVA </v>
+        <v xml:space="preserve">BADA DOST </v>
       </c>
       <c r="BQ2" t="str">
-        <v>4G</v>
+        <v>LS I4</v>
       </c>
       <c r="BR2" t="str">
-        <v/>
+        <v>MH-49-BZ-1012</v>
       </c>
       <c r="BS2" t="str">
-        <v/>
+        <v>HPH036172P</v>
       </c>
       <c r="BT2" t="str">
-        <v>2024-10</v>
+        <v>2023-06</v>
       </c>
       <c r="BV2" t="str">
-        <v>2024</v>
+        <v>2023</v>
       </c>
       <c r="BW2" t="str">
-        <v/>
+        <v>MB1AB42E6PRHK6364</v>
       </c>
       <c r="BX2" t="str">
         <v/>
@@ -935,13 +935,13 @@
         <v>ONLINE</v>
       </c>
       <c r="CH2">
-        <v>753</v>
+        <v>20690</v>
       </c>
       <c r="CI2" t="str">
         <v/>
       </c>
       <c r="CJ2" s="1">
-        <v>45837</v>
+        <v>46214</v>
       </c>
       <c r="CK2" t="str">
         <v/>
@@ -962,22 +962,25 @@
         <v>0</v>
       </c>
       <c r="CQ2">
-        <v>25</v>
+        <v>19.5</v>
       </c>
       <c r="CR2">
-        <v>9.75</v>
+        <v>895.25</v>
       </c>
       <c r="CS2">
-        <v>25</v>
+        <v>37.5</v>
       </c>
       <c r="CT2">
-        <v>178.5</v>
+        <v>6037.13</v>
       </c>
       <c r="CU2">
-        <v>188.25</v>
+        <v>6932.38</v>
+      </c>
+      <c r="CV2">
+        <v>18</v>
       </c>
       <c r="CW2">
-        <v>188.25</v>
+        <v>8180.21</v>
       </c>
     </row>
     <row r="3">
@@ -985,10 +988,10 @@
         <v>2026-2027</v>
       </c>
       <c r="B3" t="str">
-        <v>retail</v>
+        <v>RETAIL</v>
       </c>
       <c r="C3" t="str">
-        <v>SURESH</v>
+        <v>MANSI SHARMA</v>
       </c>
       <c r="D3" t="str">
         <v/>
@@ -1000,246 +1003,1651 @@
         <v/>
       </c>
       <c r="G3" t="str">
-        <v>test</v>
+        <v>JP INSURANCE BROKERS PVT LTD</v>
       </c>
       <c r="H3" t="str">
-        <v>test</v>
+        <v>NAGPUR</v>
       </c>
       <c r="I3" t="str">
+        <v>MRS</v>
+      </c>
+      <c r="J3" t="str">
+        <v>MANSI SHARMA</v>
+      </c>
+      <c r="K3" t="str">
+        <v>9999999999</v>
+      </c>
+      <c r="L3" t="str">
+        <v>test@gmail.com</v>
+      </c>
+      <c r="M3" t="str">
+        <v>SHRIRAM GENERAL INSURANCE CO. LTD</v>
+      </c>
+      <c r="N3" t="str">
+        <v>54678956789</v>
+      </c>
+      <c r="O3" t="b">
+        <v>0</v>
+      </c>
+      <c r="P3" t="str">
+        <v/>
+      </c>
+      <c r="Q3" t="str">
+        <v/>
+      </c>
+      <c r="R3" t="str">
+        <v/>
+      </c>
+      <c r="S3" t="str">
+        <v>MOTOR</v>
+      </c>
+      <c r="T3" t="str">
+        <v>FLEXI BHARAT SOOKSHMA UDYAM</v>
+      </c>
+      <c r="U3" t="str">
+        <v/>
+      </c>
+      <c r="V3" t="str">
+        <v>SHRIRAM GENERAL INSURANCE CO. LTD</v>
+      </c>
+      <c r="W3" t="str">
+        <v>JP INSURANCE BROKER PVT. LTD</v>
+      </c>
+      <c r="X3" t="str">
+        <v>NAGPUR</v>
+      </c>
+      <c r="Y3" t="str">
+        <v>YEARLY</v>
+      </c>
+      <c r="Z3" s="1">
+        <v>46225</v>
+      </c>
+      <c r="AA3" s="1">
+        <v>46589</v>
+      </c>
+      <c r="AB3" t="str">
+        <v>1000</v>
+      </c>
+      <c r="AC3">
+        <v>9</v>
+      </c>
+      <c r="AD3" t="str">
+        <v>90</v>
+      </c>
+      <c r="AE3" t="str">
+        <v>1090</v>
+      </c>
+      <c r="AF3" t="str">
+        <v>YEARLY</v>
+      </c>
+      <c r="AG3" s="1">
+        <v>46226</v>
+      </c>
+      <c r="AH3" s="1">
+        <v>46590</v>
+      </c>
+      <c r="AI3" t="str">
+        <v>1000</v>
+      </c>
+      <c r="AJ3">
+        <v>9</v>
+      </c>
+      <c r="AK3" t="str">
+        <v>90</v>
+      </c>
+      <c r="AL3" t="str">
+        <v>1090</v>
+      </c>
+      <c r="AM3" t="str">
+        <v>PL55</v>
+      </c>
+      <c r="AN3" s="1">
+        <v>46590</v>
+      </c>
+      <c r="AP3" t="str">
+        <v/>
+      </c>
+      <c r="AQ3" t="str">
+        <v/>
+      </c>
+      <c r="AR3" t="str">
+        <v/>
+      </c>
+      <c r="AS3" t="str">
+        <v/>
+      </c>
+      <c r="AT3" t="str">
+        <v/>
+      </c>
+      <c r="AU3" s="1">
+        <v>46226</v>
+      </c>
+      <c r="AV3" s="1">
+        <v>46590</v>
+      </c>
+      <c r="AW3" t="str">
+        <v/>
+      </c>
+      <c r="AX3" t="str">
+        <v/>
+      </c>
+      <c r="AY3" t="str">
+        <v/>
+      </c>
+      <c r="AZ3">
+        <v>2000</v>
+      </c>
+      <c r="BA3" t="str">
+        <v/>
+      </c>
+      <c r="BB3" t="str">
+        <v/>
+      </c>
+      <c r="BC3" t="str">
+        <v/>
+      </c>
+      <c r="BD3" t="str">
+        <v/>
+      </c>
+      <c r="BE3" t="str">
+        <v/>
+      </c>
+      <c r="BF3">
+        <v>180</v>
+      </c>
+      <c r="BG3" t="str">
+        <v>2180</v>
+      </c>
+      <c r="BH3" t="str">
+        <v/>
+      </c>
+      <c r="BI3" t="str">
+        <v/>
+      </c>
+      <c r="BJ3" t="str">
+        <v/>
+      </c>
+      <c r="BK3" t="str">
+        <v/>
+      </c>
+      <c r="BL3" t="str">
+        <v/>
+      </c>
+      <c r="BM3" t="str">
+        <v/>
+      </c>
+      <c r="BN3" t="str">
+        <v/>
+      </c>
+      <c r="BO3" t="str">
+        <v/>
+      </c>
+      <c r="BP3" t="str">
+        <v/>
+      </c>
+      <c r="BQ3" t="str">
+        <v/>
+      </c>
+      <c r="BR3" t="str">
+        <v/>
+      </c>
+      <c r="BS3" t="str">
+        <v/>
+      </c>
+      <c r="BT3" t="str">
+        <v/>
+      </c>
+      <c r="BU3" t="str">
+        <v/>
+      </c>
+      <c r="BV3" t="str">
+        <v/>
+      </c>
+      <c r="BW3" t="str">
+        <v/>
+      </c>
+      <c r="BX3" t="str">
+        <v/>
+      </c>
+      <c r="BY3" t="str">
+        <v/>
+      </c>
+      <c r="BZ3" t="str">
+        <v/>
+      </c>
+      <c r="CC3" t="str">
+        <v/>
+      </c>
+      <c r="CD3" t="str">
+        <v/>
+      </c>
+      <c r="CF3" t="str">
+        <v/>
+      </c>
+      <c r="CH3">
+        <v>2180</v>
+      </c>
+      <c r="CI3" t="str">
+        <v/>
+      </c>
+      <c r="CJ3" s="1">
+        <v>46224</v>
+      </c>
+      <c r="CK3" t="str">
+        <v/>
+      </c>
+      <c r="CL3" t="str">
+        <v/>
+      </c>
+      <c r="CM3" t="str">
+        <v/>
+      </c>
+      <c r="CN3">
+        <v>0</v>
+      </c>
+      <c r="CO3" t="str">
+        <v/>
+      </c>
+      <c r="CP3">
+        <v>0</v>
+      </c>
+      <c r="CQ3" t="str">
+        <v/>
+      </c>
+      <c r="CR3">
+        <v>0</v>
+      </c>
+      <c r="CS3" t="str">
+        <v/>
+      </c>
+      <c r="CT3">
+        <v>0</v>
+      </c>
+      <c r="CU3">
+        <v>0</v>
+      </c>
+      <c r="CW3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>2026-2027</v>
+      </c>
+      <c r="B4" t="str">
+        <v>RETAIL</v>
+      </c>
+      <c r="C4" t="str">
+        <v>KJHUYG</v>
+      </c>
+      <c r="D4" t="str">
+        <v/>
+      </c>
+      <c r="E4" t="str">
+        <v/>
+      </c>
+      <c r="F4" t="str">
+        <v/>
+      </c>
+      <c r="G4" t="str">
+        <v>180000</v>
+      </c>
+      <c r="H4" t="str">
+        <v>ARUN</v>
+      </c>
+      <c r="I4" t="str">
         <v>Mr.</v>
       </c>
-      <c r="J3" t="str">
-        <v>SURESH</v>
-      </c>
-      <c r="K3" t="str">
-        <v>960904445</v>
-      </c>
-      <c r="L3" t="str">
-        <v/>
-      </c>
-      <c r="M3" t="str">
+      <c r="J4" t="str">
+        <v>KJHUYG</v>
+      </c>
+      <c r="K4" t="str">
+        <v/>
+      </c>
+      <c r="L4" t="str">
+        <v/>
+      </c>
+      <c r="M4" t="str">
+        <v>ACKO GENERAL INSURANCE LIMITED</v>
+      </c>
+      <c r="N4" t="str">
+        <v/>
+      </c>
+      <c r="O4" t="b">
+        <v>0</v>
+      </c>
+      <c r="P4" t="str">
+        <v/>
+      </c>
+      <c r="Q4" t="str">
+        <v/>
+      </c>
+      <c r="R4" t="str">
+        <v/>
+      </c>
+      <c r="S4" t="str">
+        <v>ENGINEERING</v>
+      </c>
+      <c r="T4" t="str">
+        <v>TRAILERS LIABILITY</v>
+      </c>
+      <c r="U4" t="str">
+        <v/>
+      </c>
+      <c r="V4" t="str">
+        <v>ACKO GENERAL INSURANCE LIMITED</v>
+      </c>
+      <c r="W4" t="str">
+        <v>JP INSURANCE BROKER PVT. LTD</v>
+      </c>
+      <c r="X4" t="str">
+        <v>NAGPUR</v>
+      </c>
+      <c r="Y4" t="str">
+        <v/>
+      </c>
+      <c r="AB4" t="str">
+        <v/>
+      </c>
+      <c r="AC4" t="str">
+        <v/>
+      </c>
+      <c r="AD4" t="str">
+        <v>0</v>
+      </c>
+      <c r="AE4" t="str">
+        <v>0</v>
+      </c>
+      <c r="AF4" t="str">
+        <v/>
+      </c>
+      <c r="AI4" t="str">
+        <v/>
+      </c>
+      <c r="AJ4" t="str">
+        <v/>
+      </c>
+      <c r="AK4" t="str">
+        <v>0</v>
+      </c>
+      <c r="AL4" t="str">
+        <v>0</v>
+      </c>
+      <c r="AM4" t="str">
+        <v>JHJGHVJK</v>
+      </c>
+      <c r="AP4" t="str">
+        <v/>
+      </c>
+      <c r="AQ4" t="str">
+        <v/>
+      </c>
+      <c r="AR4" t="str">
+        <v/>
+      </c>
+      <c r="AS4" t="str">
+        <v/>
+      </c>
+      <c r="AT4" t="str">
+        <v/>
+      </c>
+      <c r="AW4" t="str">
+        <v/>
+      </c>
+      <c r="AX4" t="str">
+        <v/>
+      </c>
+      <c r="AY4" t="str">
+        <v/>
+      </c>
+      <c r="AZ4">
+        <v>0</v>
+      </c>
+      <c r="BA4" t="str">
+        <v/>
+      </c>
+      <c r="BB4" t="str">
+        <v/>
+      </c>
+      <c r="BC4" t="str">
+        <v/>
+      </c>
+      <c r="BD4" t="str">
+        <v/>
+      </c>
+      <c r="BE4" t="str">
+        <v/>
+      </c>
+      <c r="BF4">
+        <v>0</v>
+      </c>
+      <c r="BG4" t="str">
+        <v/>
+      </c>
+      <c r="BH4" t="str">
+        <v/>
+      </c>
+      <c r="BI4" t="str">
+        <v/>
+      </c>
+      <c r="BJ4" t="str">
+        <v/>
+      </c>
+      <c r="BK4" t="str">
+        <v/>
+      </c>
+      <c r="BL4" t="str">
+        <v/>
+      </c>
+      <c r="BM4" t="str">
+        <v/>
+      </c>
+      <c r="BN4" t="str">
+        <v/>
+      </c>
+      <c r="BO4" t="str">
+        <v/>
+      </c>
+      <c r="BP4" t="str">
+        <v/>
+      </c>
+      <c r="BQ4" t="str">
+        <v/>
+      </c>
+      <c r="BR4" t="str">
+        <v/>
+      </c>
+      <c r="BS4" t="str">
+        <v/>
+      </c>
+      <c r="BT4" t="str">
+        <v/>
+      </c>
+      <c r="BU4" t="str">
+        <v/>
+      </c>
+      <c r="BV4" t="str">
+        <v/>
+      </c>
+      <c r="BW4" t="str">
+        <v/>
+      </c>
+      <c r="BX4" t="str">
+        <v/>
+      </c>
+      <c r="BY4" t="str">
+        <v/>
+      </c>
+      <c r="BZ4" t="str">
+        <v/>
+      </c>
+      <c r="CC4" t="str">
+        <v/>
+      </c>
+      <c r="CD4" t="str">
+        <v/>
+      </c>
+      <c r="CF4" t="str">
+        <v/>
+      </c>
+      <c r="CH4">
+        <v>0</v>
+      </c>
+      <c r="CI4" t="str">
+        <v/>
+      </c>
+      <c r="CK4" t="str">
+        <v/>
+      </c>
+      <c r="CL4" t="str">
+        <v/>
+      </c>
+      <c r="CM4" t="str">
+        <v/>
+      </c>
+      <c r="CO4" t="str">
+        <v/>
+      </c>
+      <c r="CQ4" t="str">
+        <v/>
+      </c>
+      <c r="CS4" t="str">
+        <v/>
+      </c>
+      <c r="CW4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>2026-2027</v>
+      </c>
+      <c r="B5" t="str">
+        <v>RETAIL</v>
+      </c>
+      <c r="C5" t="str">
+        <v>NARESH KUMAR BANSAL</v>
+      </c>
+      <c r="D5" t="str">
+        <v/>
+      </c>
+      <c r="E5" t="str">
+        <v/>
+      </c>
+      <c r="F5" t="str">
+        <v/>
+      </c>
+      <c r="G5" t="str">
+        <v>JP INSURANCE BROKERS PVT LTD</v>
+      </c>
+      <c r="H5" t="str">
+        <v>NAGPUR</v>
+      </c>
+      <c r="I5" t="str">
+        <v>Mr.</v>
+      </c>
+      <c r="J5" t="str">
+        <v>NARESH KUMAR BANSAL</v>
+      </c>
+      <c r="K5" t="str">
+        <v>9310155845</v>
+      </c>
+      <c r="L5" t="str">
+        <v>daditrading2019@gmail.com</v>
+      </c>
+      <c r="M5" t="str">
+        <v>GENERALI CENTRAL INSURANCE COMPANY LIMITED</v>
+      </c>
+      <c r="N5" t="str">
+        <v/>
+      </c>
+      <c r="O5" t="b">
+        <v>0</v>
+      </c>
+      <c r="P5" t="str">
+        <v/>
+      </c>
+      <c r="Q5" t="str">
+        <v/>
+      </c>
+      <c r="R5" t="str">
+        <v/>
+      </c>
+      <c r="S5" t="str">
+        <v>FIRE</v>
+      </c>
+      <c r="T5" t="str">
+        <v>BHARAT SOOKSHMA LITE</v>
+      </c>
+      <c r="U5" t="str">
+        <v/>
+      </c>
+      <c r="V5" t="str">
+        <v>GENERALI CENTRAL INSURANCE COMPANY LIMITED</v>
+      </c>
+      <c r="W5" t="str">
+        <v>JP INSURANCE BROKER PVT. LTD</v>
+      </c>
+      <c r="X5" t="str">
+        <v>NAGPUR</v>
+      </c>
+      <c r="Y5" t="str">
+        <v/>
+      </c>
+      <c r="AB5" t="str">
+        <v/>
+      </c>
+      <c r="AC5" t="str">
+        <v/>
+      </c>
+      <c r="AD5" t="str">
+        <v>0</v>
+      </c>
+      <c r="AE5" t="str">
+        <v>0</v>
+      </c>
+      <c r="AF5" t="str">
+        <v/>
+      </c>
+      <c r="AI5" t="str">
+        <v/>
+      </c>
+      <c r="AJ5" t="str">
+        <v/>
+      </c>
+      <c r="AK5" t="str">
+        <v>0</v>
+      </c>
+      <c r="AL5" t="str">
+        <v>0</v>
+      </c>
+      <c r="AM5" t="str">
+        <v>132/00/00/0627/FUS/0000397831</v>
+      </c>
+      <c r="AN5" s="1">
+        <v>46561</v>
+      </c>
+      <c r="AP5" t="str">
+        <v>RENEWAL</v>
+      </c>
+      <c r="AQ5" t="str">
+        <v/>
+      </c>
+      <c r="AR5" t="str">
+        <v/>
+      </c>
+      <c r="AS5" t="str">
+        <v/>
+      </c>
+      <c r="AT5" t="str">
+        <v>YEARLY</v>
+      </c>
+      <c r="AU5" s="1">
+        <v>46197</v>
+      </c>
+      <c r="AV5" s="1">
+        <v>46561</v>
+      </c>
+      <c r="AW5" t="str">
+        <v/>
+      </c>
+      <c r="AX5" t="str">
+        <v/>
+      </c>
+      <c r="AY5" t="str">
+        <v/>
+      </c>
+      <c r="AZ5">
+        <v>6230</v>
+      </c>
+      <c r="BA5" t="str">
+        <v/>
+      </c>
+      <c r="BB5" t="str">
+        <v/>
+      </c>
+      <c r="BC5" t="str">
+        <v/>
+      </c>
+      <c r="BD5" t="str">
+        <v/>
+      </c>
+      <c r="BE5">
+        <v>18</v>
+      </c>
+      <c r="BF5">
+        <v>1121.4</v>
+      </c>
+      <c r="BG5" t="str">
+        <v>7351.4</v>
+      </c>
+      <c r="BH5" t="str">
+        <v/>
+      </c>
+      <c r="BI5" t="str">
+        <v/>
+      </c>
+      <c r="BJ5" t="str">
+        <v/>
+      </c>
+      <c r="BK5" t="str">
+        <v/>
+      </c>
+      <c r="BL5" t="str">
+        <v/>
+      </c>
+      <c r="BM5" t="str">
+        <v/>
+      </c>
+      <c r="BN5" t="str">
+        <v>6230</v>
+      </c>
+      <c r="BO5" t="str">
+        <v/>
+      </c>
+      <c r="BP5" t="str">
+        <v/>
+      </c>
+      <c r="BQ5" t="str">
+        <v/>
+      </c>
+      <c r="BR5" t="str">
+        <v/>
+      </c>
+      <c r="BS5" t="str">
+        <v/>
+      </c>
+      <c r="BT5" t="str">
+        <v/>
+      </c>
+      <c r="BU5" t="str">
+        <v/>
+      </c>
+      <c r="BV5" t="str">
+        <v/>
+      </c>
+      <c r="BW5" t="str">
+        <v/>
+      </c>
+      <c r="BX5" t="str">
+        <v/>
+      </c>
+      <c r="BY5" t="str">
+        <v/>
+      </c>
+      <c r="BZ5" t="str">
+        <v/>
+      </c>
+      <c r="CC5" t="str">
+        <v/>
+      </c>
+      <c r="CD5" t="str">
+        <v/>
+      </c>
+      <c r="CF5" t="str">
+        <v>ONLINE</v>
+      </c>
+      <c r="CH5">
+        <v>7351.4</v>
+      </c>
+      <c r="CI5" t="str">
+        <v/>
+      </c>
+      <c r="CJ5" s="1">
+        <v>46195</v>
+      </c>
+      <c r="CK5" t="str">
+        <v/>
+      </c>
+      <c r="CL5" t="str">
+        <v/>
+      </c>
+      <c r="CM5">
+        <v>30</v>
+      </c>
+      <c r="CN5">
+        <v>1869</v>
+      </c>
+      <c r="CO5" t="str">
+        <v/>
+      </c>
+      <c r="CP5">
+        <v>0</v>
+      </c>
+      <c r="CQ5" t="str">
+        <v/>
+      </c>
+      <c r="CS5" t="str">
+        <v/>
+      </c>
+      <c r="CU5">
+        <v>1869</v>
+      </c>
+      <c r="CW5">
+        <v>1869</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>2026-2027</v>
+      </c>
+      <c r="B6" t="str">
+        <v>RETAIL</v>
+      </c>
+      <c r="C6" t="str">
+        <v>FNVHBFN</v>
+      </c>
+      <c r="D6" t="str">
+        <v/>
+      </c>
+      <c r="E6" t="str">
+        <v/>
+      </c>
+      <c r="F6" t="str">
+        <v/>
+      </c>
+      <c r="G6" t="str">
+        <v>180000</v>
+      </c>
+      <c r="H6" t="str">
+        <v>ARUN</v>
+      </c>
+      <c r="I6" t="str">
+        <v>Mr.</v>
+      </c>
+      <c r="J6" t="str">
+        <v>FNVHBFN</v>
+      </c>
+      <c r="K6" t="str">
+        <v/>
+      </c>
+      <c r="L6" t="str">
+        <v>djvnj</v>
+      </c>
+      <c r="M6" t="str">
+        <v>NAVI GENERAL INSURANCE</v>
+      </c>
+      <c r="N6" t="str">
+        <v>5454586586</v>
+      </c>
+      <c r="O6" t="b">
+        <v>0</v>
+      </c>
+      <c r="P6" t="str">
+        <v/>
+      </c>
+      <c r="Q6" t="str">
+        <v/>
+      </c>
+      <c r="R6" t="str">
+        <v/>
+      </c>
+      <c r="S6" t="str">
+        <v>MOTOR</v>
+      </c>
+      <c r="T6" t="str">
+        <v>FLEXI GRIHA RAKSHA</v>
+      </c>
+      <c r="U6" t="str">
+        <v/>
+      </c>
+      <c r="V6" t="str">
+        <v>NAVI GENERAL INSURANCE</v>
+      </c>
+      <c r="W6" t="str">
+        <v>JP INSURANCE BROKER PVT. LTD</v>
+      </c>
+      <c r="X6" t="str">
+        <v>NAGPUR</v>
+      </c>
+      <c r="Y6" t="str">
+        <v>YEARLY</v>
+      </c>
+      <c r="Z6" s="1">
+        <v>46225</v>
+      </c>
+      <c r="AA6" s="1">
+        <v>46589</v>
+      </c>
+      <c r="AB6" t="str">
+        <v>10000</v>
+      </c>
+      <c r="AC6">
+        <v>18</v>
+      </c>
+      <c r="AD6" t="str">
+        <v>1800</v>
+      </c>
+      <c r="AE6" t="str">
+        <v>11800</v>
+      </c>
+      <c r="AF6" t="str">
+        <v>YEARLY</v>
+      </c>
+      <c r="AG6" s="1">
+        <v>46226</v>
+      </c>
+      <c r="AH6" s="1">
+        <v>46590</v>
+      </c>
+      <c r="AI6" t="str">
+        <v>10000</v>
+      </c>
+      <c r="AJ6">
+        <v>18</v>
+      </c>
+      <c r="AK6" t="str">
+        <v>1800</v>
+      </c>
+      <c r="AL6" t="str">
+        <v>11800</v>
+      </c>
+      <c r="AM6" t="str">
+        <v>SDJF</v>
+      </c>
+      <c r="AN6" s="1">
+        <v>46590</v>
+      </c>
+      <c r="AP6" t="str">
+        <v/>
+      </c>
+      <c r="AQ6" t="str">
+        <v/>
+      </c>
+      <c r="AR6" t="str">
+        <v/>
+      </c>
+      <c r="AS6" t="str">
+        <v/>
+      </c>
+      <c r="AT6" t="str">
+        <v/>
+      </c>
+      <c r="AU6" s="1">
+        <v>46226</v>
+      </c>
+      <c r="AV6" s="1">
+        <v>46590</v>
+      </c>
+      <c r="AW6" t="str">
+        <v/>
+      </c>
+      <c r="AX6" t="str">
+        <v/>
+      </c>
+      <c r="AY6" t="str">
+        <v/>
+      </c>
+      <c r="AZ6">
+        <v>20000</v>
+      </c>
+      <c r="BA6" t="str">
+        <v/>
+      </c>
+      <c r="BB6" t="str">
+        <v/>
+      </c>
+      <c r="BC6" t="str">
+        <v/>
+      </c>
+      <c r="BD6" t="str">
+        <v/>
+      </c>
+      <c r="BE6" t="str">
+        <v/>
+      </c>
+      <c r="BF6">
+        <v>3600</v>
+      </c>
+      <c r="BG6" t="str">
+        <v>23600</v>
+      </c>
+      <c r="BH6" t="str">
+        <v/>
+      </c>
+      <c r="BI6" t="str">
+        <v/>
+      </c>
+      <c r="BJ6" t="str">
+        <v/>
+      </c>
+      <c r="BK6" t="str">
+        <v/>
+      </c>
+      <c r="BL6" t="str">
+        <v/>
+      </c>
+      <c r="BM6" t="str">
+        <v/>
+      </c>
+      <c r="BN6" t="str">
+        <v/>
+      </c>
+      <c r="BO6" t="str">
+        <v/>
+      </c>
+      <c r="BP6" t="str">
+        <v/>
+      </c>
+      <c r="BQ6" t="str">
+        <v/>
+      </c>
+      <c r="BR6" t="str">
+        <v/>
+      </c>
+      <c r="BS6" t="str">
+        <v/>
+      </c>
+      <c r="BT6" t="str">
+        <v/>
+      </c>
+      <c r="BU6" t="str">
+        <v/>
+      </c>
+      <c r="BV6" t="str">
+        <v/>
+      </c>
+      <c r="BW6" t="str">
+        <v/>
+      </c>
+      <c r="BX6" t="str">
+        <v/>
+      </c>
+      <c r="BZ6" t="str">
+        <v/>
+      </c>
+      <c r="CC6" t="str">
+        <v/>
+      </c>
+      <c r="CD6" t="str">
+        <v/>
+      </c>
+      <c r="CF6" t="str">
+        <v/>
+      </c>
+      <c r="CH6">
+        <v>23600</v>
+      </c>
+      <c r="CI6" t="str">
+        <v/>
+      </c>
+      <c r="CJ6" s="1">
+        <v>46224</v>
+      </c>
+      <c r="CK6" t="str">
+        <v/>
+      </c>
+      <c r="CL6" t="str">
+        <v/>
+      </c>
+      <c r="CM6" t="str">
+        <v/>
+      </c>
+      <c r="CN6">
+        <v>0</v>
+      </c>
+      <c r="CO6" t="str">
+        <v/>
+      </c>
+      <c r="CP6">
+        <v>0</v>
+      </c>
+      <c r="CQ6" t="str">
+        <v/>
+      </c>
+      <c r="CR6">
+        <v>0</v>
+      </c>
+      <c r="CS6" t="str">
+        <v/>
+      </c>
+      <c r="CT6">
+        <v>0</v>
+      </c>
+      <c r="CU6">
+        <v>0</v>
+      </c>
+      <c r="CW6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>2026-2027</v>
+      </c>
+      <c r="B7" t="str">
+        <v>RETAIL</v>
+      </c>
+      <c r="C7" t="str">
+        <v>MEGHRAJ TOLARAM MAINANI</v>
+      </c>
+      <c r="D7" t="str">
+        <v/>
+      </c>
+      <c r="E7" t="str">
+        <v/>
+      </c>
+      <c r="F7" t="str">
+        <v/>
+      </c>
+      <c r="G7" t="str">
+        <v>JP INSURANCE BROKERS PVT LTD</v>
+      </c>
+      <c r="H7" t="str">
+        <v>NAGPUR</v>
+      </c>
+      <c r="I7" t="str">
+        <v>Mr.</v>
+      </c>
+      <c r="J7" t="str">
+        <v>MEGHRAJ TOLARAM MAINANI</v>
+      </c>
+      <c r="K7" t="str">
+        <v>9822226753</v>
+      </c>
+      <c r="L7" t="str">
+        <v>skmohak@yahoo.com</v>
+      </c>
+      <c r="M7" t="str">
         <v>TATA AIG GENERAL INSURANCE CO. LTD</v>
       </c>
-      <c r="N3" t="str">
-        <v/>
-      </c>
-      <c r="O3" t="b">
-        <v>0</v>
-      </c>
-      <c r="P3" t="str">
-        <v/>
-      </c>
-      <c r="Q3" t="str">
-        <v/>
-      </c>
-      <c r="R3" t="str">
-        <v/>
-      </c>
-      <c r="S3" t="str">
-        <v>HEALTH</v>
-      </c>
-      <c r="T3" t="str">
-        <v>MY HEALTH CARE - FLOATER</v>
-      </c>
-      <c r="U3" t="str">
-        <v/>
-      </c>
-      <c r="V3" t="str">
-        <v/>
-      </c>
-      <c r="W3" t="str">
-        <v>test</v>
-      </c>
-      <c r="X3" t="str">
-        <v>test</v>
-      </c>
-      <c r="Y3" t="str">
-        <v/>
-      </c>
-      <c r="AB3" t="str">
-        <v/>
-      </c>
-      <c r="AC3" t="str">
-        <v/>
-      </c>
-      <c r="AD3" t="str">
-        <v>0</v>
-      </c>
-      <c r="AE3" t="str">
-        <v>0</v>
-      </c>
-      <c r="AF3" t="str">
-        <v/>
-      </c>
-      <c r="AI3" t="str">
-        <v/>
-      </c>
-      <c r="AJ3" t="str">
-        <v/>
-      </c>
-      <c r="AK3" t="str">
-        <v>0</v>
-      </c>
-      <c r="AL3" t="str">
-        <v>0</v>
-      </c>
-      <c r="AM3" t="str">
-        <v>123456987</v>
-      </c>
-      <c r="AN3" s="1">
-        <v>46568</v>
-      </c>
-      <c r="AO3">
-        <v>1000000</v>
-      </c>
-      <c r="AP3" t="str">
+      <c r="N7" t="str">
+        <v/>
+      </c>
+      <c r="O7" t="b">
+        <v>0</v>
+      </c>
+      <c r="P7" t="str">
+        <v/>
+      </c>
+      <c r="Q7" t="str">
+        <v/>
+      </c>
+      <c r="R7" t="str">
+        <v/>
+      </c>
+      <c r="S7" t="str">
+        <v>MOTOR</v>
+      </c>
+      <c r="T7" t="str">
+        <v>CAR</v>
+      </c>
+      <c r="U7" t="str">
+        <v/>
+      </c>
+      <c r="V7" t="str">
+        <v>TATA AIG GENERAL INSURANCE CO. LTD</v>
+      </c>
+      <c r="W7" t="str">
+        <v>JP INSURANCE BROKER PVT. LTD</v>
+      </c>
+      <c r="X7" t="str">
+        <v>NAGPUR</v>
+      </c>
+      <c r="Y7" t="str">
+        <v>YEARLY</v>
+      </c>
+      <c r="Z7" s="1">
+        <v>46213</v>
+      </c>
+      <c r="AA7" s="1">
+        <v>46577</v>
+      </c>
+      <c r="AB7" t="str">
+        <v>8672</v>
+      </c>
+      <c r="AC7">
+        <v>18</v>
+      </c>
+      <c r="AD7" t="str">
+        <v>1560.96</v>
+      </c>
+      <c r="AE7" t="str">
+        <v>10232.96</v>
+      </c>
+      <c r="AF7" t="str">
+        <v>YEARLY</v>
+      </c>
+      <c r="AG7" s="1">
+        <v>46213</v>
+      </c>
+      <c r="AH7" s="1">
+        <v>46577</v>
+      </c>
+      <c r="AI7" t="str">
+        <v>3238</v>
+      </c>
+      <c r="AJ7">
+        <v>18</v>
+      </c>
+      <c r="AK7" t="str">
+        <v>582.84</v>
+      </c>
+      <c r="AL7" t="str">
+        <v>3820.84</v>
+      </c>
+      <c r="AM7" t="str">
+        <v>6201716670</v>
+      </c>
+      <c r="AN7" s="1">
+        <v>46577</v>
+      </c>
+      <c r="AO7">
+        <v>1490400</v>
+      </c>
+      <c r="AP7" t="str">
         <v>RENEWAL</v>
       </c>
-      <c r="AQ3" t="str">
-        <v/>
-      </c>
-      <c r="AR3" t="str">
-        <v/>
-      </c>
-      <c r="AT3" t="str">
+      <c r="AQ7" t="str">
+        <v/>
+      </c>
+      <c r="AR7" t="str">
+        <v/>
+      </c>
+      <c r="AS7" t="str">
+        <v/>
+      </c>
+      <c r="AT7" t="str">
+        <v/>
+      </c>
+      <c r="AW7" t="str">
+        <v/>
+      </c>
+      <c r="AX7" t="str">
+        <v/>
+      </c>
+      <c r="AY7" t="str">
+        <v/>
+      </c>
+      <c r="AZ7">
+        <v>11910</v>
+      </c>
+      <c r="BA7" t="str">
+        <v/>
+      </c>
+      <c r="BB7" t="str">
+        <v/>
+      </c>
+      <c r="BC7" t="str">
+        <v/>
+      </c>
+      <c r="BD7" t="str">
+        <v/>
+      </c>
+      <c r="BE7" t="str">
+        <v/>
+      </c>
+      <c r="BF7">
+        <v>2143.8</v>
+      </c>
+      <c r="BG7" t="str">
+        <v>14053.8</v>
+      </c>
+      <c r="BH7" t="str">
+        <v/>
+      </c>
+      <c r="BI7" t="str">
+        <v/>
+      </c>
+      <c r="BJ7" t="str">
+        <v/>
+      </c>
+      <c r="BK7" t="str">
+        <v/>
+      </c>
+      <c r="BL7" t="str">
+        <v/>
+      </c>
+      <c r="BM7" t="str">
+        <v/>
+      </c>
+      <c r="BN7" t="str">
+        <v/>
+      </c>
+      <c r="BO7" t="str">
+        <v xml:space="preserve">TOYOTA </v>
+      </c>
+      <c r="BP7" t="str">
+        <v xml:space="preserve">INNOVA CRY STA </v>
+      </c>
+      <c r="BQ7" t="str">
+        <v>2.4 GX MT 7 STR</v>
+      </c>
+      <c r="BR7" t="str">
+        <v>MH 49 BW 9071</v>
+      </c>
+      <c r="BS7" t="str">
+        <v>2GDA730169</v>
+      </c>
+      <c r="BT7" t="str">
+        <v>2023-06</v>
+      </c>
+      <c r="BV7" t="str">
+        <v>2023</v>
+      </c>
+      <c r="BW7" t="str">
+        <v>MBJJB8EM4016413560623</v>
+      </c>
+      <c r="BX7" t="str">
+        <v/>
+      </c>
+      <c r="BY7" t="str">
+        <v/>
+      </c>
+      <c r="BZ7" t="str">
+        <v/>
+      </c>
+      <c r="CC7" t="str">
+        <v/>
+      </c>
+      <c r="CD7" t="str">
+        <v/>
+      </c>
+      <c r="CF7" t="str">
+        <v>ONLINE</v>
+      </c>
+      <c r="CG7">
+        <v>0</v>
+      </c>
+      <c r="CH7">
+        <v>14053.8</v>
+      </c>
+      <c r="CI7" t="str">
+        <v/>
+      </c>
+      <c r="CJ7" s="1">
+        <v>46211</v>
+      </c>
+      <c r="CK7" t="str">
+        <v/>
+      </c>
+      <c r="CL7" t="str">
+        <v/>
+      </c>
+      <c r="CM7" t="str">
+        <v/>
+      </c>
+      <c r="CN7">
+        <v>0</v>
+      </c>
+      <c r="CO7" t="str">
+        <v/>
+      </c>
+      <c r="CP7">
+        <v>0</v>
+      </c>
+      <c r="CQ7">
+        <v>25</v>
+      </c>
+      <c r="CR7">
+        <v>809.5</v>
+      </c>
+      <c r="CS7" t="str">
+        <v/>
+      </c>
+      <c r="CT7">
+        <v>0</v>
+      </c>
+      <c r="CU7">
+        <v>809.5</v>
+      </c>
+      <c r="CW7">
+        <v>809.5</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>2026-2027</v>
+      </c>
+      <c r="B8" t="str">
+        <v>RETAIL</v>
+      </c>
+      <c r="C8" t="str">
+        <v>ANSHUL AGRAWAL</v>
+      </c>
+      <c r="D8" t="str">
+        <v/>
+      </c>
+      <c r="E8" t="str">
+        <v/>
+      </c>
+      <c r="F8" t="str">
+        <v/>
+      </c>
+      <c r="G8" t="str">
+        <v>JP INSURANCE BROKERS PVT LTD</v>
+      </c>
+      <c r="H8" t="str">
+        <v>NAGPUR</v>
+      </c>
+      <c r="I8" t="str">
+        <v>Mr.</v>
+      </c>
+      <c r="J8" t="str">
+        <v>ANSHUL AGRAWAL</v>
+      </c>
+      <c r="K8" t="str">
+        <v>8888770000</v>
+      </c>
+      <c r="L8" t="str">
+        <v/>
+      </c>
+      <c r="M8" t="str">
+        <v>TATA AIG GENERAL INSURANCE CO. LTD</v>
+      </c>
+      <c r="N8" t="str">
+        <v/>
+      </c>
+      <c r="O8" t="b">
+        <v>0</v>
+      </c>
+      <c r="P8" t="str">
+        <v/>
+      </c>
+      <c r="Q8" t="str">
+        <v/>
+      </c>
+      <c r="R8" t="str">
+        <v/>
+      </c>
+      <c r="S8" t="str">
+        <v>MOTOR</v>
+      </c>
+      <c r="T8" t="str">
+        <v>CAR</v>
+      </c>
+      <c r="U8" t="str">
+        <v/>
+      </c>
+      <c r="V8" t="str">
+        <v>TATA AIG GENERAL INSURANCE CO. LTD</v>
+      </c>
+      <c r="W8" t="str">
+        <v>JP INSURANCE BROKER PVT. LTD</v>
+      </c>
+      <c r="X8" t="str">
+        <v>NAGPUR</v>
+      </c>
+      <c r="Y8" t="str">
         <v>YEARLY</v>
       </c>
-      <c r="AU3" s="1">
-        <v>46204</v>
-      </c>
-      <c r="AV3" s="1">
-        <v>46568</v>
-      </c>
-      <c r="AW3" t="str">
-        <v/>
-      </c>
-      <c r="AY3" t="str">
-        <v/>
-      </c>
-      <c r="AZ3">
-        <v>12000</v>
-      </c>
-      <c r="BA3" t="str">
-        <v/>
-      </c>
-      <c r="BB3" t="str">
-        <v/>
-      </c>
-      <c r="BC3" t="str">
-        <v/>
-      </c>
-      <c r="BD3" t="str">
-        <v/>
-      </c>
-      <c r="BE3" t="str">
-        <v/>
-      </c>
-      <c r="BF3">
-        <v>0</v>
-      </c>
-      <c r="BG3" t="str">
-        <v>12000</v>
-      </c>
-      <c r="BH3" t="str">
-        <v/>
-      </c>
-      <c r="BI3" t="str">
-        <v/>
-      </c>
-      <c r="BJ3" t="str">
-        <v/>
-      </c>
-      <c r="BL3" t="str">
-        <v/>
-      </c>
-      <c r="BM3" t="str">
-        <v/>
-      </c>
-      <c r="BN3" t="str">
-        <v>12000</v>
-      </c>
-      <c r="BO3" t="str">
-        <v/>
-      </c>
-      <c r="BP3" t="str">
-        <v/>
-      </c>
-      <c r="BQ3" t="str">
-        <v/>
-      </c>
-      <c r="BR3" t="str">
-        <v/>
-      </c>
-      <c r="BS3" t="str">
-        <v/>
-      </c>
-      <c r="BT3" t="str">
-        <v/>
-      </c>
-      <c r="BV3" t="str">
-        <v/>
-      </c>
-      <c r="BW3" t="str">
-        <v/>
-      </c>
-      <c r="BX3" t="str">
-        <v/>
-      </c>
-      <c r="BZ3" t="str">
-        <v/>
-      </c>
-      <c r="CC3" t="str">
-        <v/>
-      </c>
-      <c r="CD3" t="str">
-        <v/>
-      </c>
-      <c r="CF3" t="str">
+      <c r="Z8" s="1">
+        <v>46210</v>
+      </c>
+      <c r="AA8" s="1">
+        <v>46574</v>
+      </c>
+      <c r="AB8" t="str">
+        <v>21026.11</v>
+      </c>
+      <c r="AC8">
+        <v>18</v>
+      </c>
+      <c r="AD8" t="str">
+        <v>3784.7</v>
+      </c>
+      <c r="AE8" t="str">
+        <v>24810.81</v>
+      </c>
+      <c r="AF8" t="str">
+        <v>YEARLY</v>
+      </c>
+      <c r="AG8" s="1">
+        <v>46210</v>
+      </c>
+      <c r="AH8" s="1">
+        <v>46574</v>
+      </c>
+      <c r="AI8" t="str">
+        <v>8572</v>
+      </c>
+      <c r="AJ8">
+        <v>18</v>
+      </c>
+      <c r="AK8" t="str">
+        <v>1542.96</v>
+      </c>
+      <c r="AL8" t="str">
+        <v>10114.96</v>
+      </c>
+      <c r="AM8" t="str">
+        <v>6203096011 02 00</v>
+      </c>
+      <c r="AN8" s="1">
+        <v>46574</v>
+      </c>
+      <c r="AO8">
+        <v>5324750</v>
+      </c>
+      <c r="AP8" t="str">
+        <v>RENEWAL</v>
+      </c>
+      <c r="AQ8" t="str">
+        <v/>
+      </c>
+      <c r="AR8" t="str">
+        <v/>
+      </c>
+      <c r="AS8" t="str">
+        <v/>
+      </c>
+      <c r="AT8" t="str">
+        <v/>
+      </c>
+      <c r="AU8" s="1">
+        <v>46210</v>
+      </c>
+      <c r="AV8" s="1">
+        <v>46574</v>
+      </c>
+      <c r="AW8" t="str">
+        <v/>
+      </c>
+      <c r="AX8" t="str">
+        <v/>
+      </c>
+      <c r="AY8" t="str">
+        <v/>
+      </c>
+      <c r="AZ8">
+        <v>29598.11</v>
+      </c>
+      <c r="BA8" t="str">
+        <v/>
+      </c>
+      <c r="BB8" t="str">
+        <v/>
+      </c>
+      <c r="BC8" t="str">
+        <v/>
+      </c>
+      <c r="BD8" t="str">
+        <v/>
+      </c>
+      <c r="BE8" t="str">
+        <v/>
+      </c>
+      <c r="BF8">
+        <v>5327.66</v>
+      </c>
+      <c r="BG8" t="str">
+        <v>34925.77</v>
+      </c>
+      <c r="BH8" t="str">
+        <v/>
+      </c>
+      <c r="BI8" t="str">
+        <v/>
+      </c>
+      <c r="BJ8" t="str">
+        <v/>
+      </c>
+      <c r="BK8" t="str">
+        <v/>
+      </c>
+      <c r="BL8" t="str">
+        <v/>
+      </c>
+      <c r="BM8" t="str">
+        <v/>
+      </c>
+      <c r="BN8" t="str">
+        <v>29,598.11</v>
+      </c>
+      <c r="BO8" t="str">
+        <v>JEEP /</v>
+      </c>
+      <c r="BP8" t="str">
+        <v xml:space="preserve"> GRAND CHEROK EE </v>
+      </c>
+      <c r="BQ8" t="str">
+        <v>/ SRT PETROL</v>
+      </c>
+      <c r="BR8" t="str">
+        <v>DN 09 M 2875</v>
+      </c>
+      <c r="BS8" t="str">
+        <v>6170710617</v>
+      </c>
+      <c r="BT8" t="str">
+        <v>2018-02</v>
+      </c>
+      <c r="BV8" t="str">
+        <v>2018</v>
+      </c>
+      <c r="BW8" t="str">
+        <v>1C4RJFHJ7HC9661207H</v>
+      </c>
+      <c r="BX8" t="str">
+        <v/>
+      </c>
+      <c r="BY8" t="str">
+        <v/>
+      </c>
+      <c r="BZ8" t="str">
+        <v/>
+      </c>
+      <c r="CC8" t="str">
+        <v/>
+      </c>
+      <c r="CD8" t="str">
+        <v/>
+      </c>
+      <c r="CF8" t="str">
         <v>ONLINE</v>
       </c>
-      <c r="CH3">
-        <v>12000</v>
-      </c>
-      <c r="CI3" t="str">
-        <v/>
-      </c>
-      <c r="CJ3" s="1">
-        <v>46202</v>
-      </c>
-      <c r="CK3" t="str">
-        <v/>
-      </c>
-      <c r="CL3" t="str">
-        <v/>
-      </c>
-      <c r="CM3">
-        <v>17.5</v>
-      </c>
-      <c r="CN3">
-        <v>2100</v>
-      </c>
-      <c r="CO3" t="str">
-        <v/>
-      </c>
-      <c r="CP3">
-        <v>0</v>
-      </c>
-      <c r="CQ3" t="str">
-        <v/>
-      </c>
-      <c r="CS3" t="str">
-        <v/>
-      </c>
-      <c r="CU3">
-        <v>2100</v>
-      </c>
-      <c r="CW3">
-        <v>2100</v>
+      <c r="CG8">
+        <v>0</v>
+      </c>
+      <c r="CH8">
+        <v>34925.77</v>
+      </c>
+      <c r="CI8" t="str">
+        <v/>
+      </c>
+      <c r="CJ8" s="1">
+        <v>46208</v>
+      </c>
+      <c r="CK8" t="str">
+        <v/>
+      </c>
+      <c r="CL8" t="str">
+        <v/>
+      </c>
+      <c r="CM8" t="str">
+        <v/>
+      </c>
+      <c r="CN8">
+        <v>0</v>
+      </c>
+      <c r="CO8" t="str">
+        <v/>
+      </c>
+      <c r="CP8">
+        <v>0</v>
+      </c>
+      <c r="CQ8">
+        <v>25.5</v>
+      </c>
+      <c r="CR8">
+        <v>2185.86</v>
+      </c>
+      <c r="CS8" t="str">
+        <v/>
+      </c>
+      <c r="CT8">
+        <v>0</v>
+      </c>
+      <c r="CU8">
+        <v>2185.86</v>
+      </c>
+      <c r="CW8">
+        <v>2185.86</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:CW3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:CW8"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>